<commit_message>
Completed test plan conversion code integration into rest of system
</commit_message>
<xml_diff>
--- a/Example_Test_Recipe.xlsx
+++ b/Example_Test_Recipe.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/08500da1c505d51b/Desktop/Senior Design/Team-108-Generation-of-Synthetic-Battery-Gas-for-Fire-and-Explosion-Testing-/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Devin\School\Senior Design\Team-108-Generation-of-Synthetic-Battery-Gas-for-Fire-and-Explosion-Testing-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7893C657-E207-4CF8-98A8-1C7CA93FFE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BE28EC0-B5B1-480D-B816-87485B017A1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{2CE868BB-4CDE-422B-A877-E4D21E68C372}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CE868BB-4CDE-422B-A877-E4D21E68C372}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>Time (s)</t>
   </si>
@@ -56,9 +56,6 @@
     <t>CH4</t>
   </si>
   <si>
-    <t>N2</t>
-  </si>
-  <si>
     <t>Heat Release Rate (kW)</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
   </si>
   <si>
     <t>CH4 SLPM</t>
-  </si>
-  <si>
-    <t>N2 SLPM</t>
   </si>
   <si>
     <t>Heat of Combustion (kJ/kg)</t>
@@ -103,6 +97,7 @@
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -110,6 +105,7 @@
       <sz val="11"/>
       <color theme="0"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -131,7 +127,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -169,23 +165,72 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -205,10 +250,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -528,18 +569,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1205A373-0027-4370-B8D0-F88183E8D924}">
-  <dimension ref="A1:N18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" customWidth="1"/>
-    <col min="8" max="8" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.54296875" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
-    <col min="11" max="12" width="13.81640625" customWidth="1"/>
-    <col min="13" max="13" width="14.1796875" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" customWidth="1"/>
+    <col min="10" max="11" width="13.85546875" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -558,13 +599,13 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J1" s="4" t="s">
@@ -576,14 +617,8 @@
       <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="2" spans="1:12" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>1</v>
@@ -600,20 +635,16 @@
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="5"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
       <c r="I2" s="5"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-    </row>
-    <row r="3" spans="1:14" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" ht="46.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1">
         <v>141584</v>
@@ -630,20 +661,16 @@
       <c r="F3" s="1">
         <v>55514</v>
       </c>
-      <c r="G3" s="1">
-        <v>0</v>
-      </c>
-      <c r="H3" s="5"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
       <c r="I3" s="5"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-    </row>
-    <row r="4" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" spans="1:12" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1">
         <v>8.9899999999999994E-2</v>
@@ -660,18 +687,14 @@
       <c r="F4" s="1">
         <v>1.1779999999999999</v>
       </c>
-      <c r="G4" s="1">
-        <v>1.2490000000000001</v>
-      </c>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>0</v>
       </c>
@@ -691,31 +714,27 @@
         <v>1</v>
       </c>
       <c r="G5" s="3">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H5" s="3">
-        <v>100</v>
+        <f>(B5*(G5/$B$3)*60000)/$B$4</f>
+        <v>0</v>
       </c>
       <c r="I5" s="3">
-        <f>(B5*(H5/$B$3)*60000)/$B$4</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="3">
-        <f>(C5*(H5/$C$3)*60000)/$C$4</f>
-        <v>0</v>
-      </c>
-      <c r="K5" s="3"/>
+        <f>(C5*(G5/$C$3)*60000)/$C$4</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3">
+        <f>(E5*(G5/$E$3)*60000)/$E$4</f>
+        <v>0</v>
+      </c>
       <c r="L5" s="3">
-        <f>(E5*(H5/$E$3)*60000)/$E$4</f>
-        <v>0</v>
-      </c>
-      <c r="M5" s="3">
-        <f>(F5*(H5/$F$3)*60000)/$F$4</f>
+        <f>(F5*(G5/$F$3)*60000)/$F$4</f>
         <v>91.749443524333458</v>
       </c>
-      <c r="N5" s="3"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>1</v>
       </c>
@@ -735,31 +754,27 @@
         <v>0.2</v>
       </c>
       <c r="G6" s="3">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H6" s="3">
-        <v>30</v>
+        <f>(B6*(G6/$B$3)*60000)/$B$4</f>
+        <v>28.28320564618263</v>
       </c>
       <c r="I6" s="3">
-        <f t="shared" ref="I6:I18" si="0">(B6*(H6/$B$3)*60000)/$B$4</f>
-        <v>28.28320564618263</v>
-      </c>
-      <c r="J6" s="3">
-        <f t="shared" ref="J6:J18" si="1">(C6*(H6/$C$3)*60000)/$C$4</f>
+        <f>(C6*(G6/$C$3)*60000)/$C$4</f>
         <v>31.117426796253465</v>
       </c>
-      <c r="K6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3">
+        <f>(E6*(G6/$E$3)*60000)/$E$4</f>
+        <v>4.9938564468245286</v>
+      </c>
       <c r="L6" s="3">
-        <f t="shared" ref="L6:L18" si="2">(E6*(H6/$E$3)*60000)/$E$4</f>
-        <v>4.9938564468245286</v>
-      </c>
-      <c r="M6" s="3">
-        <f t="shared" ref="M6:M17" si="3">(F6*(H6/$F$3)*60000)/$F$4</f>
+        <f>(F6*(G6/$F$3)*60000)/$F$4</f>
         <v>5.5049666114600075</v>
       </c>
-      <c r="N6" s="3"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>2</v>
       </c>
@@ -779,31 +794,27 @@
         <v>0.2</v>
       </c>
       <c r="G7" s="3">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H7" s="3">
-        <v>50</v>
+        <f>(B7*(G7/$B$3)*60000)/$B$4</f>
+        <v>70.708014115456578</v>
       </c>
       <c r="I7" s="3">
-        <f t="shared" si="0"/>
-        <v>70.708014115456578</v>
-      </c>
-      <c r="J7" s="3">
-        <f t="shared" si="1"/>
+        <f>(C7*(G7/$C$3)*60000)/$C$4</f>
         <v>25.931188996877882</v>
       </c>
-      <c r="K7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3">
+        <f>(E7*(G7/$E$3)*60000)/$E$4</f>
+        <v>8.3230940780408815</v>
+      </c>
       <c r="L7" s="3">
-        <f t="shared" si="2"/>
-        <v>8.3230940780408815</v>
-      </c>
-      <c r="M7" s="3">
-        <f t="shared" si="3"/>
+        <f>(F7*(G7/$F$3)*60000)/$F$4</f>
         <v>9.1749443524333465</v>
       </c>
-      <c r="N7" s="3"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>3</v>
       </c>
@@ -823,31 +834,27 @@
         <v>0.2</v>
       </c>
       <c r="G8" s="3">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H8" s="3">
-        <v>50</v>
+        <f>(B8*(G8/$B$3)*60000)/$B$4</f>
+        <v>58.923345096213815</v>
       </c>
       <c r="I8" s="3">
-        <f t="shared" si="0"/>
-        <v>58.923345096213815</v>
-      </c>
-      <c r="J8" s="3">
-        <f t="shared" si="1"/>
+        <f>(C8*(G8/$C$3)*60000)/$C$4</f>
         <v>25.931188996877882</v>
       </c>
-      <c r="K8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3">
+        <f>(E8*(G8/$E$3)*60000)/$E$4</f>
+        <v>8.3230940780408815</v>
+      </c>
       <c r="L8" s="3">
-        <f t="shared" si="2"/>
-        <v>8.3230940780408815</v>
-      </c>
-      <c r="M8" s="3">
-        <f t="shared" si="3"/>
+        <f>(F8*(G8/$F$3)*60000)/$F$4</f>
         <v>9.1749443524333465</v>
       </c>
-      <c r="N8" s="3"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>4</v>
       </c>
@@ -867,31 +874,27 @@
         <v>0.2</v>
       </c>
       <c r="G9" s="3">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H9" s="3">
-        <v>50</v>
+        <f>(B9*(G9/$B$3)*60000)/$B$4</f>
+        <v>47.138676076971052</v>
       </c>
       <c r="I9" s="3">
-        <f t="shared" si="0"/>
-        <v>47.138676076971052</v>
-      </c>
-      <c r="J9" s="3">
-        <f t="shared" si="1"/>
+        <f>(C9*(G9/$C$3)*60000)/$C$4</f>
         <v>25.931188996877882</v>
       </c>
-      <c r="K9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3">
+        <f>(E9*(G9/$E$3)*60000)/$E$4</f>
+        <v>8.3230940780408815</v>
+      </c>
       <c r="L9" s="3">
-        <f t="shared" si="2"/>
-        <v>8.3230940780408815</v>
-      </c>
-      <c r="M9" s="3">
-        <f t="shared" si="3"/>
+        <f>(F9*(G9/$F$3)*60000)/$F$4</f>
         <v>9.1749443524333465</v>
       </c>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>5</v>
       </c>
@@ -911,31 +914,27 @@
         <v>0.2</v>
       </c>
       <c r="G10" s="3">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H10" s="3">
-        <v>50</v>
+        <f>(B10*(G10/$B$3)*60000)/$B$4</f>
+        <v>35.354007057728289</v>
       </c>
       <c r="I10" s="3">
-        <f t="shared" si="0"/>
-        <v>35.354007057728289</v>
-      </c>
-      <c r="J10" s="3">
-        <f t="shared" si="1"/>
+        <f>(C10*(G10/$C$3)*60000)/$C$4</f>
         <v>25.931188996877882</v>
       </c>
-      <c r="K10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3">
+        <f>(E10*(G10/$E$3)*60000)/$E$4</f>
+        <v>8.3230940780408815</v>
+      </c>
       <c r="L10" s="3">
-        <f t="shared" si="2"/>
-        <v>8.3230940780408815</v>
-      </c>
-      <c r="M10" s="3">
-        <f t="shared" si="3"/>
+        <f>(F10*(G10/$F$3)*60000)/$F$4</f>
         <v>9.1749443524333465</v>
       </c>
-      <c r="N10" s="3"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>6</v>
       </c>
@@ -955,31 +954,27 @@
         <v>0.2</v>
       </c>
       <c r="G11" s="3">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H11" s="3">
-        <v>50</v>
+        <f>(B11*(G11/$B$3)*60000)/$B$4</f>
+        <v>23.569338038485526</v>
       </c>
       <c r="I11" s="3">
-        <f t="shared" si="0"/>
-        <v>23.569338038485526</v>
-      </c>
-      <c r="J11" s="3">
-        <f t="shared" si="1"/>
+        <f>(C11*(G11/$C$3)*60000)/$C$4</f>
         <v>25.931188996877882</v>
       </c>
-      <c r="K11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3">
+        <f>(E11*(G11/$E$3)*60000)/$E$4</f>
+        <v>8.3230940780408815</v>
+      </c>
       <c r="L11" s="3">
-        <f t="shared" si="2"/>
-        <v>8.3230940780408815</v>
-      </c>
-      <c r="M11" s="3">
-        <f t="shared" si="3"/>
+        <f>(F11*(G11/$F$3)*60000)/$F$4</f>
         <v>9.1749443524333465</v>
       </c>
-      <c r="N11" s="3"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>7</v>
       </c>
@@ -999,31 +994,27 @@
         <v>0.2</v>
       </c>
       <c r="G12" s="3">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H12" s="3">
-        <v>75</v>
+        <f>(B12*(G12/$B$3)*60000)/$B$4</f>
+        <v>35.354007057728289</v>
       </c>
       <c r="I12" s="3">
-        <f t="shared" si="0"/>
-        <v>35.354007057728289</v>
-      </c>
-      <c r="J12" s="3">
-        <f t="shared" si="1"/>
+        <f>(C12*(G12/$C$3)*60000)/$C$4</f>
         <v>38.896783495316825</v>
       </c>
-      <c r="K12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3">
+        <f>(E12*(G12/$E$3)*60000)/$E$4</f>
+        <v>12.484641117061324</v>
+      </c>
       <c r="L12" s="3">
-        <f t="shared" si="2"/>
-        <v>12.484641117061324</v>
-      </c>
-      <c r="M12" s="3">
-        <f t="shared" si="3"/>
+        <f>(F12*(G12/$F$3)*60000)/$F$4</f>
         <v>13.762416528650016</v>
       </c>
-      <c r="N12" s="3"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>8</v>
       </c>
@@ -1043,31 +1034,27 @@
         <v>0.2</v>
       </c>
       <c r="G13" s="3">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H13" s="3">
-        <v>75</v>
+        <f>(B13*(G13/$B$3)*60000)/$B$4</f>
+        <v>35.354007057728289</v>
       </c>
       <c r="I13" s="3">
-        <f t="shared" si="0"/>
-        <v>35.354007057728289</v>
-      </c>
-      <c r="J13" s="3">
-        <f t="shared" si="1"/>
+        <f>(C13*(G13/$C$3)*60000)/$C$4</f>
         <v>38.896783495316825</v>
       </c>
-      <c r="K13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3">
+        <f>(E13*(G13/$E$3)*60000)/$E$4</f>
+        <v>0</v>
+      </c>
       <c r="L13" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M13" s="3">
-        <f t="shared" si="3"/>
+        <f>(F13*(G13/$F$3)*60000)/$F$4</f>
         <v>13.762416528650016</v>
       </c>
-      <c r="N13" s="3"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>9</v>
       </c>
@@ -1087,31 +1074,27 @@
         <v>0.2</v>
       </c>
       <c r="G14" s="3">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H14" s="3">
-        <v>75</v>
+        <f>(B14*(G14/$B$3)*60000)/$B$4</f>
+        <v>0</v>
       </c>
       <c r="I14" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J14" s="3">
-        <f t="shared" si="1"/>
+        <f>(C14*(G14/$C$3)*60000)/$C$4</f>
         <v>38.896783495316825</v>
       </c>
-      <c r="K14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3">
+        <f>(E14*(G14/$E$3)*60000)/$E$4</f>
+        <v>12.484641117061324</v>
+      </c>
       <c r="L14" s="3">
-        <f t="shared" si="2"/>
-        <v>12.484641117061324</v>
-      </c>
-      <c r="M14" s="3">
-        <f t="shared" si="3"/>
+        <f>(F14*(G14/$F$3)*60000)/$F$4</f>
         <v>13.762416528650016</v>
       </c>
-      <c r="N14" s="3"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>10</v>
       </c>
@@ -1131,31 +1114,27 @@
         <v>0.2</v>
       </c>
       <c r="G15" s="3">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H15" s="3">
-        <v>75</v>
+        <f>(B15*(G15/$B$3)*60000)/$B$4</f>
+        <v>0</v>
       </c>
       <c r="I15" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J15" s="3">
-        <f t="shared" si="1"/>
+        <f>(C15*(G15/$C$3)*60000)/$C$4</f>
         <v>38.896783495316825</v>
       </c>
-      <c r="K15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3">
+        <f>(E15*(G15/$E$3)*60000)/$E$4</f>
+        <v>12.484641117061324</v>
+      </c>
       <c r="L15" s="3">
-        <f t="shared" si="2"/>
-        <v>12.484641117061324</v>
-      </c>
-      <c r="M15" s="3">
-        <f t="shared" si="3"/>
+        <f>(F15*(G15/$F$3)*60000)/$F$4</f>
         <v>13.762416528650016</v>
       </c>
-      <c r="N15" s="3"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>11</v>
       </c>
@@ -1175,31 +1154,27 @@
         <v>0.2</v>
       </c>
       <c r="G16" s="3">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H16" s="3">
-        <v>75</v>
+        <f>(B16*(G16/$B$3)*60000)/$B$4</f>
+        <v>176.77003528864142</v>
       </c>
       <c r="I16" s="3">
-        <f t="shared" si="0"/>
-        <v>176.77003528864142</v>
-      </c>
-      <c r="J16" s="3">
-        <f t="shared" si="1"/>
+        <f>(C16*(G16/$C$3)*60000)/$C$4</f>
         <v>38.896783495316825</v>
       </c>
-      <c r="K16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3">
+        <f>(E16*(G16/$E$3)*60000)/$E$4</f>
+        <v>12.484641117061324</v>
+      </c>
       <c r="L16" s="3">
-        <f t="shared" si="2"/>
-        <v>12.484641117061324</v>
-      </c>
-      <c r="M16" s="3">
-        <f t="shared" si="3"/>
+        <f>(F16*(G16/$F$3)*60000)/$F$4</f>
         <v>13.762416528650016</v>
       </c>
-      <c r="N16" s="3"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>13</v>
       </c>
@@ -1219,31 +1194,27 @@
         <v>0.2</v>
       </c>
       <c r="G17" s="3">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H17" s="3">
-        <v>75</v>
+        <f>(B17*(G17/$B$3)*60000)/$B$4</f>
+        <v>0</v>
       </c>
       <c r="I17" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J17" s="3">
-        <f t="shared" si="1"/>
+        <f>(C17*(G17/$C$3)*60000)/$C$4</f>
         <v>38.896783495316825</v>
       </c>
-      <c r="K17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3">
+        <f>(E17*(G17/$E$3)*60000)/$E$4</f>
+        <v>12.484641117061324</v>
+      </c>
       <c r="L17" s="3">
-        <f t="shared" si="2"/>
-        <v>12.484641117061324</v>
-      </c>
-      <c r="M17" s="3">
-        <f t="shared" si="3"/>
+        <f>(F17*(G17/$F$3)*60000)/$F$4</f>
         <v>13.762416528650016</v>
       </c>
-      <c r="N17" s="3"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>15</v>
       </c>
@@ -1266,36 +1237,31 @@
         <v>0</v>
       </c>
       <c r="H18" s="3">
+        <f>(B18*(G18/$B$3)*60000)/$B$4</f>
         <v>0</v>
       </c>
       <c r="I18" s="3">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J18" s="3">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K18" s="3"/>
+        <f>(C18*(G18/$C$3)*60000)/$C$4</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3">
+        <f>(E18*(G18/$E$3)*60000)/$E$4</f>
+        <v>0</v>
+      </c>
       <c r="L18" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M18" s="3">
-        <f t="shared" ref="M18" si="4">(F18*(H18/$F$3)*60000)/$F$4</f>
-        <v>0</v>
-      </c>
-      <c r="N18" s="3"/>
+        <f>(F18*(G18/$F$3)*60000)/$F$4</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="N1:N4"/>
+  <mergeCells count="6">
+    <mergeCell ref="G1:G4"/>
     <mergeCell ref="H1:H4"/>
     <mergeCell ref="I1:I4"/>
     <mergeCell ref="J1:J4"/>
     <mergeCell ref="K1:K4"/>
     <mergeCell ref="L1:L4"/>
-    <mergeCell ref="M1:M4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>